<commit_message>
Add the audit and QA evidence, design-review screenshots, main-server configuration notes, local-testing helper scripts, old migration bundles, the store master and vendor e-mail workbooks, and the latest performance run results (no passwords, keys or tokens; audit-stack temp secrets and local-password files are left out)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/VENDOR-EMAIL-MAP.xlsx
+++ b/docs/VENDOR-EMAIL-MAP.xlsx
@@ -1,18 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29127"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{637DB4E4-95E1-47A7-B30E-D4F5C47005B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Mail map" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="Who gets what" state="visible" r:id="rId5"/>
+    <sheet name="Mail map" sheetId="1" r:id="rId1"/>
+    <sheet name="Who gets what" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="143">
   <si>
     <t>Vendor journey - who gets which e-mail, when, with what words, and where the address comes from (checked 2026-10-23)</t>
   </si>
@@ -423,37 +427,65 @@
   </si>
   <si>
     <t>Mail 1 created; Mail 4 assigned; every status change (5, 6, 7, 8, 9, 13, 18, 24); Mail 10 vendor message; Mail 21 cancelled; Mail 25 resolved with rating links; Mail 26 reminder; Mail 29 reopened. NOT mailed for revised-price requests, revised quotes, or a quote rejected while the ticket goes on.</t>
+  </si>
+  <si>
+    <t>Here also email should shoot to store, by saying Parts list updated and show the updated list in mail also and converstaion is added with part list</t>
+  </si>
+  <si>
+    <t>Didn’t understand explain this in simple language</t>
+  </si>
+  <si>
+    <t>if we remove this Po approver and add PO Approver in AC Master sheet? And if we add 2 emails then it will go to 2 approvers and it we add 1 then it goes to 1 approver. And each store and each ac have that approver email address as we have now in mail to column? Whats your suggestion?</t>
+  </si>
+  <si>
+    <t>didn’t understandneed to understand ythis in detail. As in above point mail triggered when quote was rejected now what is here? Its rejection of ticket only? And worrding is also not seems good as I understood once you make me understand proper then we can suggets wording</t>
+  </si>
+  <si>
+    <t>here vendor should see its reopened.</t>
+  </si>
+  <si>
+    <t>Our Remarks</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="5" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
       <sz val="13"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
       <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="12"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -490,8 +522,14 @@
         <fgColor rgb="FFE8F5E9"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -514,17 +552,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB0B7C3"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB0B7C3"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -544,10 +591,19 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -886,9 +942,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G40"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:H40"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
     <col min="2" max="2" width="44" customWidth="1"/>
@@ -897,882 +953,914 @@
     <col min="5" max="5" width="44" customWidth="1"/>
     <col min="6" max="6" width="70" customWidth="1"/>
     <col min="7" max="7" width="62" customWidth="1"/>
+    <col min="8" max="8" width="8.88671875" style="13"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:8" ht="17.399999999999999" x14ac:dyDescent="0.35">
+      <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
+      <c r="F1" s="10"/>
+      <c r="G1" s="10"/>
+    </row>
+    <row r="2" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="1" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
+      <c r="H2" s="15" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A3" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
+      <c r="B3" s="11"/>
+      <c r="C3" s="11"/>
+      <c r="D3" s="11"/>
+      <c r="E3" s="11"/>
+      <c r="F3" s="11"/>
+      <c r="G3" s="11"/>
+    </row>
+    <row r="4" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E4" s="5" t="s">
+      <c r="D4" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="F4" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="G4" s="5" t="s">
+      <c r="G4" s="3" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
+    <row r="5" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E5" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="F5" s="5" t="s">
+      <c r="F5" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="G5" s="5" t="s">
+      <c r="G5" s="3" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="4" t="s">
+    <row r="6" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="C6" s="8" t="s">
+      <c r="C6" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="D6" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E6" s="5" t="s">
+      <c r="D6" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="F6" s="5" t="s">
+      <c r="F6" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="G6" s="5" t="s">
+      <c r="G6" s="3" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
+    <row r="7" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D7" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E7" s="5" t="s">
+      <c r="D7" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E7" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="F7" s="5" t="s">
+      <c r="F7" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="G7" s="5" t="s">
+      <c r="G7" s="3" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
+    <row r="8" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A8" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="B8" s="3"/>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
-      <c r="E8" s="3"/>
-      <c r="F8" s="3"/>
-      <c r="G8" s="3"/>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="4" t="s">
+      <c r="B8" s="11"/>
+      <c r="C8" s="11"/>
+      <c r="D8" s="11"/>
+      <c r="E8" s="11"/>
+      <c r="F8" s="11"/>
+      <c r="G8" s="11"/>
+    </row>
+    <row r="9" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="C9" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D9" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E9" s="5" t="s">
+      <c r="D9" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E9" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="F9" s="5" t="s">
+      <c r="F9" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="G9" s="5" t="s">
+      <c r="G9" s="3" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="4" t="s">
+    <row r="10" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A10" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="C10" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D10" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E10" s="5" t="s">
+      <c r="D10" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E10" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="F10" s="5" t="s">
+      <c r="F10" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="G10" s="5" t="s">
+      <c r="G10" s="3" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" s="4" t="s">
+    <row r="11" spans="1:8" ht="273.60000000000002" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="C11" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="D11" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="F11" s="5" t="s">
+      <c r="D11" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F11" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="G11" s="5" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="4" t="s">
+      <c r="G11" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="H11" s="14" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="B12" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="C12" s="6" t="s">
+      <c r="C12" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D12" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E12" s="5" t="s">
+      <c r="D12" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E12" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="F12" s="5" t="s">
+      <c r="F12" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="G12" s="5" t="s">
+      <c r="G12" s="3" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="4" t="s">
+    <row r="13" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A13" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="C13" s="6" t="s">
+      <c r="C13" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D13" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E13" s="5" t="s">
+      <c r="D13" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E13" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="F13" s="5" t="s">
+      <c r="F13" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="G13" s="5" t="s">
+      <c r="G13" s="3" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="4" t="s">
+    <row r="14" spans="1:8" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A14" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="B14" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="C14" s="6" t="s">
+      <c r="C14" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D14" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E14" s="5" t="s">
+      <c r="D14" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E14" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="F14" s="5" t="s">
+      <c r="F14" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="G14" s="5" t="s">
+      <c r="G14" s="3" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" s="4" t="s">
+      <c r="H14" s="14" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A15" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="B15" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="C15" s="6" t="s">
+      <c r="C15" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D15" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E15" s="5" t="s">
+      <c r="D15" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E15" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="F15" s="5" t="s">
+      <c r="F15" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="G15" s="5" t="s">
+      <c r="G15" s="3" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A16" s="4" t="s">
+    <row r="16" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A16" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B16" s="5" t="s">
+      <c r="B16" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="C16" s="8" t="s">
+      <c r="C16" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="D16" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E16" s="5" t="s">
+      <c r="D16" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E16" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="F16" s="5" t="s">
+      <c r="F16" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="G16" s="5" t="s">
+      <c r="G16" s="3" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="3" t="s">
+    <row r="17" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A17" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="B17" s="3"/>
-      <c r="C17" s="3"/>
-      <c r="D17" s="3"/>
-      <c r="E17" s="3"/>
-      <c r="F17" s="3"/>
-      <c r="G17" s="3"/>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="4" t="s">
+      <c r="B17" s="11"/>
+      <c r="C17" s="11"/>
+      <c r="D17" s="11"/>
+      <c r="E17" s="11"/>
+      <c r="F17" s="11"/>
+      <c r="G17" s="11"/>
+    </row>
+    <row r="18" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A18" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="B18" s="5" t="s">
+      <c r="B18" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="C18" s="9" t="s">
+      <c r="C18" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="D18" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E18" s="5" t="s">
+      <c r="D18" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E18" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="F18" s="5" t="s">
+      <c r="F18" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="G18" s="5" t="s">
+      <c r="G18" s="3" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="4" t="s">
+      <c r="H18" s="14" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A19" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="B19" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="C19" s="6" t="s">
+      <c r="C19" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D19" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E19" s="5" t="s">
+      <c r="D19" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E19" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="F19" s="5" t="s">
+      <c r="F19" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="G19" s="5" t="s">
+      <c r="G19" s="3" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="4" t="s">
+    <row r="20" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A20" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="B20" s="5" t="s">
+      <c r="B20" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="C20" s="8" t="s">
+      <c r="C20" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="D20" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E20" s="5" t="s">
+      <c r="D20" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E20" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="F20" s="5" t="s">
+      <c r="F20" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="G20" s="5" t="s">
+      <c r="G20" s="3" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A21" s="4" t="s">
+    <row r="21" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A21" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="B21" s="5" t="s">
+      <c r="B21" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="C21" s="9" t="s">
+      <c r="C21" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="D21" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E21" s="5" t="s">
+      <c r="D21" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E21" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="F21" s="5" t="s">
+      <c r="F21" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="G21" s="5" t="s">
+      <c r="G21" s="3" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" s="4" t="s">
+      <c r="H21" s="14" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A22" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="B22" s="5" t="s">
+      <c r="B22" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="C22" s="7" t="s">
+      <c r="C22" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="D22" s="5" t="s">
+      <c r="D22" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="E22" s="5" t="s">
+      <c r="E22" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="F22" s="5" t="s">
+      <c r="F22" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="G22" s="5" t="s">
+      <c r="G22" s="3" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" s="4" t="s">
+      <c r="H22" s="14"/>
+    </row>
+    <row r="23" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A23" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="B23" s="5" t="s">
+      <c r="B23" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="C23" s="8" t="s">
+      <c r="C23" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="D23" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E23" s="5" t="s">
+      <c r="D23" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E23" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="F23" s="5" t="s">
+      <c r="F23" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="G23" s="5" t="s">
+      <c r="G23" s="3" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="4" t="s">
+    <row r="24" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A24" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="B24" s="5" t="s">
+      <c r="B24" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="C24" s="6" t="s">
+      <c r="C24" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D24" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E24" s="5" t="s">
+      <c r="D24" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E24" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="F24" s="5" t="s">
+      <c r="F24" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="G24" s="5" t="s">
+      <c r="G24" s="3" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" s="4" t="s">
+    <row r="25" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A25" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="B25" s="5" t="s">
+      <c r="B25" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C25" s="8" t="s">
+      <c r="C25" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="D25" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E25" s="5" t="s">
+      <c r="D25" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E25" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="F25" s="5" t="s">
+      <c r="F25" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="G25" s="5" t="s">
+      <c r="G25" s="3" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A26" s="4" t="s">
+    <row r="26" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A26" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="B26" s="5" t="s">
+      <c r="B26" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="C26" s="7" t="s">
+      <c r="C26" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="D26" s="5" t="s">
+      <c r="D26" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="E26" s="5" t="s">
+      <c r="E26" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="F26" s="5" t="s">
+      <c r="F26" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="G26" s="5" t="s">
+      <c r="G26" s="3" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="4" t="s">
+      <c r="H26" s="14" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A27" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="B27" s="5" t="s">
+      <c r="B27" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="C27" s="6" t="s">
+      <c r="C27" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D27" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E27" s="5" t="s">
+      <c r="D27" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E27" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="F27" s="5" t="s">
+      <c r="F27" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="G27" s="5" t="s">
+      <c r="G27" s="3" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" s="4" t="s">
+      <c r="H27" s="14" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A28" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="B28" s="5" t="s">
+      <c r="B28" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="C28" s="8" t="s">
+      <c r="C28" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="D28" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E28" s="5" t="s">
+      <c r="D28" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E28" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="F28" s="5" t="s">
+      <c r="F28" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="G28" s="5" t="s">
+      <c r="G28" s="3" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A29" s="4" t="s">
+      <c r="H28" s="14" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A29" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="B29" s="5" t="s">
+      <c r="B29" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="C29" s="9" t="s">
+      <c r="C29" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="D29" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E29" s="5" t="s">
+      <c r="D29" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E29" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="F29" s="5" t="s">
+      <c r="F29" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="G29" s="5" t="s">
+      <c r="G29" s="3" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30" s="4" t="s">
+      <c r="H29" s="14" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A30" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="B30" s="5" t="s">
+      <c r="B30" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="C30" s="6" t="s">
+      <c r="C30" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D30" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E30" s="5" t="s">
+      <c r="D30" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E30" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="F30" s="5" t="s">
+      <c r="F30" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="G30" s="5" t="s">
+      <c r="G30" s="3" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A31" s="3" t="s">
+    <row r="31" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A31" s="11" t="s">
         <v>108</v>
       </c>
-      <c r="B31" s="3"/>
-      <c r="C31" s="3"/>
-      <c r="D31" s="3"/>
-      <c r="E31" s="3"/>
-      <c r="F31" s="3"/>
-      <c r="G31" s="3"/>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A32" s="4" t="s">
+      <c r="B31" s="11"/>
+      <c r="C31" s="11"/>
+      <c r="D31" s="11"/>
+      <c r="E31" s="11"/>
+      <c r="F31" s="11"/>
+      <c r="G31" s="11"/>
+    </row>
+    <row r="32" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A32" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="B32" s="5" t="s">
+      <c r="B32" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="C32" s="6" t="s">
+      <c r="C32" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D32" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E32" s="5" t="s">
+      <c r="D32" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E32" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="F32" s="5" t="s">
+      <c r="F32" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="G32" s="5" t="s">
+      <c r="G32" s="3" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" s="4" t="s">
+    <row r="33" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A33" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="B33" s="5" t="s">
+      <c r="B33" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="C33" s="6" t="s">
+      <c r="C33" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D33" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E33" s="5" t="s">
+      <c r="D33" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E33" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="F33" s="5" t="s">
+      <c r="F33" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="G33" s="5" t="s">
+      <c r="G33" s="3" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A34" s="4" t="s">
+    <row r="34" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A34" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="B34" s="5" t="s">
+      <c r="B34" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="C34" s="7" t="s">
+      <c r="C34" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="D34" s="5" t="s">
+      <c r="D34" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="E34" s="5" t="s">
+      <c r="E34" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="F34" s="5" t="s">
+      <c r="F34" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="G34" s="5" t="s">
+      <c r="G34" s="3" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A35" s="4" t="s">
+    <row r="35" spans="1:8" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A35" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="B35" s="5" t="s">
+      <c r="B35" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="C35" s="8" t="s">
+      <c r="C35" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="D35" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E35" s="5" t="s">
+      <c r="D35" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E35" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="F35" s="5" t="s">
+      <c r="F35" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="G35" s="5" t="s">
+      <c r="G35" s="3" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A36" s="4" t="s">
+      <c r="H35" s="14" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A36" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="B36" s="5" t="s">
+      <c r="B36" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="C36" s="6" t="s">
+      <c r="C36" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D36" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E36" s="5" t="s">
+      <c r="D36" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E36" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="F36" s="5" t="s">
+      <c r="F36" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="G36" s="5" t="s">
+      <c r="G36" s="3" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="38" ht="32" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A38" s="10" t="s">
+    <row r="38" spans="1:8" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="8" t="s">
         <v>125</v>
       </c>
-      <c r="B38" s="11" t="s">
+      <c r="B38" s="12" t="s">
         <v>126</v>
       </c>
-      <c r="C38" s="11"/>
-      <c r="D38" s="11"/>
-      <c r="E38" s="11"/>
-      <c r="F38" s="11"/>
-      <c r="G38" s="11"/>
-    </row>
-    <row r="39" ht="32" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A39" s="10" t="s">
+      <c r="C38" s="12"/>
+      <c r="D38" s="12"/>
+      <c r="E38" s="12"/>
+      <c r="F38" s="12"/>
+      <c r="G38" s="12"/>
+    </row>
+    <row r="39" spans="1:8" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="8" t="s">
         <v>127</v>
       </c>
-      <c r="B39" s="11" t="s">
+      <c r="B39" s="12" t="s">
         <v>128</v>
       </c>
-      <c r="C39" s="11"/>
-      <c r="D39" s="11"/>
-      <c r="E39" s="11"/>
-      <c r="F39" s="11"/>
-      <c r="G39" s="11"/>
-    </row>
-    <row r="40" ht="32" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A40" s="10" t="s">
+      <c r="C39" s="12"/>
+      <c r="D39" s="12"/>
+      <c r="E39" s="12"/>
+      <c r="F39" s="12"/>
+      <c r="G39" s="12"/>
+    </row>
+    <row r="40" spans="1:8" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="8" t="s">
         <v>129</v>
       </c>
-      <c r="B40" s="11" t="s">
+      <c r="B40" s="12" t="s">
         <v>130</v>
       </c>
-      <c r="C40" s="11"/>
-      <c r="D40" s="11"/>
-      <c r="E40" s="11"/>
-      <c r="F40" s="11"/>
-      <c r="G40" s="11"/>
+      <c r="C40" s="12"/>
+      <c r="D40" s="12"/>
+      <c r="E40" s="12"/>
+      <c r="F40" s="12"/>
+      <c r="G40" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="8">
+    <mergeCell ref="B38:G38"/>
+    <mergeCell ref="B39:G39"/>
+    <mergeCell ref="B40:G40"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A3:G3"/>
     <mergeCell ref="A8:G8"/>
     <mergeCell ref="A17:G17"/>
     <mergeCell ref="A31:G31"/>
-    <mergeCell ref="B38:G38"/>
-    <mergeCell ref="B39:G39"/>
-    <mergeCell ref="B40:G40"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
     <col min="2" max="2" width="140" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="12" t="s">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" s="9" t="s">
         <v>131</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="9" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
+    <row r="2" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="3" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="3" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
+    <row r="4" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="3" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
+    <row r="5" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="3" t="s">
         <v>136</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>